<commit_message>
feat(resources): brand all workbooks and handouts to match PDF convention (P1-03)
</commit_message>
<xml_diff>
--- a/public/downloads/automation-tools/budget-pacing-dayparting-analyzer.xlsx
+++ b/public/downloads/automation-tools/budget-pacing-dayparting-analyzer.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="How to use" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Settings" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Daily Pacing" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Hourly Dayparting" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to use" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily Pacing" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hourly Dayparting" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -535,7 +535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -548,6 +548,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="42" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -583,8 +584,23 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Project Amazon PH Academy — Download Center</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;9 Project Amazon PH Academy — Download Center</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -691,6 +707,14 @@
     <mergeCell ref="A1:C1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;9 Project Amazon PH Academy — Download Center</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -892,6 +916,14 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;9 Project Amazon PH Academy — Download Center</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -1227,5 +1259,13 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;9 Project Amazon PH Academy — Download Center</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(resources): brand all workbooks and handouts to match PDF convention (P1-03) (#493)
</commit_message>
<xml_diff>
--- a/public/downloads/automation-tools/budget-pacing-dayparting-analyzer.xlsx
+++ b/public/downloads/automation-tools/budget-pacing-dayparting-analyzer.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="How to use" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Settings" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Daily Pacing" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Hourly Dayparting" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to use" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily Pacing" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hourly Dayparting" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -535,7 +535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -548,6 +548,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="42" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -583,8 +584,23 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Project Amazon PH Academy — Download Center</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;9 Project Amazon PH Academy — Download Center</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -691,6 +707,14 @@
     <mergeCell ref="A1:C1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;9 Project Amazon PH Academy — Download Center</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -892,6 +916,14 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;9 Project Amazon PH Academy — Download Center</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -1227,5 +1259,13 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;9 Project Amazon PH Academy — Download Center</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>